<commit_message>
changes to tomato excel
</commit_message>
<xml_diff>
--- a/data/crops/rothc_support/tomatoes_rothc_scenarios.xlsx
+++ b/data/crops/rothc_support/tomatoes_rothc_scenarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldwildlifefund-my.sharepoint.com/personal/cristobal_loyola_wwfus_org/Documents/Documents/203. Python projects/SBTN_Test/data/crops/rothc_support/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="198" documentId="8_{33C6C299-611E-4211-942E-822619945D17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CFE80DB2-3E0B-42E0-AA74-A649492259C4}"/>
+  <xr:revisionPtr revIDLastSave="206" documentId="8_{33C6C299-611E-4211-942E-822619945D17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E71E5A89-B7CC-4694-9B32-834C059A88C3}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6F94B64D-243B-49DA-AE87-045B34BFAB0F}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2326" uniqueCount="612">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2283" uniqueCount="614">
   <si>
     <t>crop_name</t>
   </si>
@@ -1942,12 +1942,18 @@
   <si>
     <t>../LEAFs/SOC/rasters/test</t>
   </si>
+  <si>
+    <t>apply_soc_clip</t>
+  </si>
+  <si>
+    <t>soc_global_percentile_cap</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1984,6 +1990,13 @@
     <font>
       <sz val="7"/>
       <color rgb="FFFF8B39"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="7"/>
+      <color rgb="FFFF7EDB"/>
       <name val="Consolas"/>
       <family val="3"/>
     </font>
@@ -2047,7 +2060,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2058,6 +2071,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2497,7 +2513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1821CC5-2977-4A1A-B60B-8C004F05C4AF}">
-  <dimension ref="A1:Z7"/>
+  <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.36328125" bestFit="1" customWidth="1"/>
@@ -2509,7 +2525,7 @@
     <col min="8" max="8" width="63.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2588,8 +2604,14 @@
       <c r="Z1" s="2" t="s">
         <v>608</v>
       </c>
-    </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="AA1" s="10" t="s">
+        <v>612</v>
+      </c>
+      <c r="AB1" s="10" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>32</v>
       </c>
@@ -2664,8 +2686,14 @@
       <c r="Z2" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="AA2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB2">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -2740,8 +2768,14 @@
       <c r="Z3" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="AA3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB3">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -2816,222 +2850,41 @@
       <c r="Z4" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" t="s">
-        <v>408</v>
-      </c>
-      <c r="D5" t="s">
-        <v>408</v>
-      </c>
-      <c r="E5">
-        <v>14</v>
-      </c>
-      <c r="F5" t="s">
-        <v>611</v>
-      </c>
-      <c r="G5" t="str">
-        <f t="shared" ref="G5" si="4">+"RothC results for year 2030 for "&amp;A5&amp;"_"&amp;D5&amp;" in ton C/ha"</f>
-        <v>RothC results for year 2030 for Tomato_rf in ton C/ha</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>433</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>398</v>
-      </c>
-      <c r="N5" t="b">
-        <v>0</v>
-      </c>
-      <c r="O5" t="b">
-        <v>0</v>
-      </c>
-      <c r="P5">
-        <v>100</v>
-      </c>
-      <c r="Q5" s="6" t="s">
-        <v>592</v>
-      </c>
-      <c r="R5" s="5" t="s">
-        <v>593</v>
-      </c>
-      <c r="S5" s="5" t="s">
-        <v>591</v>
-      </c>
-      <c r="T5" s="6" t="s">
-        <v>592</v>
-      </c>
-      <c r="U5" t="b">
-        <v>0</v>
-      </c>
-      <c r="V5" t="s">
-        <v>597</v>
-      </c>
-      <c r="W5" t="s">
-        <v>601</v>
-      </c>
-      <c r="X5" t="s">
-        <v>602</v>
-      </c>
-      <c r="Y5">
-        <v>0</v>
-      </c>
-      <c r="Z5" t="b">
+      <c r="AA4" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" t="s">
-        <v>408</v>
-      </c>
-      <c r="D6" t="s">
-        <v>408</v>
-      </c>
-      <c r="E6">
-        <v>14</v>
-      </c>
-      <c r="F6" t="s">
-        <v>611</v>
-      </c>
-      <c r="G6" t="str">
-        <f t="shared" ref="G6:G7" si="5">+"RothC results for year 2030 for "&amp;A6&amp;"_"&amp;D6&amp;" in ton C/ha"</f>
-        <v>RothC results for year 2030 for Tomato_rf in ton C/ha</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>433</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>398</v>
-      </c>
-      <c r="N6" t="b">
-        <v>0</v>
-      </c>
-      <c r="O6" t="b">
-        <v>0</v>
-      </c>
-      <c r="P6">
-        <v>100</v>
-      </c>
-      <c r="Q6" s="6" t="s">
-        <v>592</v>
-      </c>
-      <c r="R6" s="5" t="s">
-        <v>593</v>
-      </c>
-      <c r="S6" s="5" t="s">
-        <v>591</v>
-      </c>
-      <c r="T6" s="6" t="s">
-        <v>592</v>
-      </c>
-      <c r="U6" t="b">
-        <v>0</v>
-      </c>
-      <c r="V6" t="s">
-        <v>597</v>
-      </c>
-      <c r="W6" s="9" t="s">
-        <v>609</v>
-      </c>
-      <c r="X6" t="s">
-        <v>602</v>
-      </c>
-      <c r="Y6">
-        <v>0</v>
-      </c>
-      <c r="Z6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B7" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" t="s">
-        <v>408</v>
-      </c>
-      <c r="D7" t="s">
-        <v>408</v>
-      </c>
-      <c r="E7">
-        <v>14</v>
-      </c>
-      <c r="F7" t="s">
-        <v>611</v>
-      </c>
-      <c r="G7" t="str">
-        <f t="shared" si="5"/>
-        <v>RothC results for year 2030 for Tomato_rf in ton C/ha</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>433</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>398</v>
-      </c>
-      <c r="N7" t="b">
-        <v>0</v>
-      </c>
-      <c r="O7" t="b">
-        <v>0</v>
-      </c>
-      <c r="P7">
-        <v>100</v>
-      </c>
-      <c r="Q7" s="6" t="s">
-        <v>592</v>
-      </c>
-      <c r="R7" s="5" t="s">
-        <v>593</v>
-      </c>
-      <c r="S7" s="5" t="s">
-        <v>591</v>
-      </c>
-      <c r="T7" s="6" t="s">
-        <v>592</v>
-      </c>
-      <c r="U7" t="b">
-        <v>0</v>
-      </c>
-      <c r="V7" t="s">
-        <v>597</v>
-      </c>
-      <c r="W7" s="9" t="s">
-        <v>610</v>
-      </c>
-      <c r="X7" t="s">
-        <v>602</v>
-      </c>
-      <c r="Y7">
-        <v>2</v>
-      </c>
-      <c r="Z7" t="b">
-        <v>1</v>
-      </c>
+      <c r="AB4">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="4"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="5"/>
+      <c r="S5" s="5"/>
+      <c r="T5" s="6"/>
+    </row>
+    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="4"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="5"/>
+      <c r="S6" s="5"/>
+      <c r="T6" s="6"/>
+      <c r="W6" s="9"/>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="4"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="5"/>
+      <c r="S7" s="5"/>
+      <c r="T7" s="6"/>
+      <c r="W7" s="9"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:T24" xr:uid="{A1821CC5-2977-4A1A-B60B-8C004F05C4AF}"/>

</xml_diff>